<commit_message>
corrigindo funcionalidade de cruzamento de planilha de vendas
</commit_message>
<xml_diff>
--- a/planilhasParaCruzamento/Fechamento Fev26 a Maio26 Vivo (1).xlsx
+++ b/planilhasParaCruzamento/Fechamento Fev26 a Maio26 Vivo (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USERs\Documents\GitHub\pos-venda\planilhasParaCruzamento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB728219-EFD3-431E-85B8-22B1EE2B0D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172A8024-073F-4D98-8CFA-A9C596E2DC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4740" yWindow="2580" windowWidth="22815" windowHeight="12375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4170" yWindow="2340" windowWidth="22815" windowHeight="12375" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FEVEREIRO26" sheetId="1" r:id="rId1"/>

</xml_diff>